<commit_message>
Fix Imperial section detection; red only for non-BEK items before Imperial
- Detect Imperial divider by bek_num == 'Imperial' (was broken before)
- Items in Imperial section: no red, price-change colors only
- Items before Imperial with no BEK# or wrong BEK#: solid stop-sign red
- Simplified to one red color for all unmatched items (no orange split)
- 48 pre-Imperial items need manual BEK lookup; 32 Imperial items clean

https://claude.ai/code/session_01X8paGHaWL7mkyS14PYXe6Z
</commit_message>
<xml_diff>
--- a/Updated_185_Count_Sheet_BEK_v2.xlsx
+++ b/Updated_185_Count_Sheet_BEK_v2.xlsx
@@ -75,12 +75,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF6600"/>
+        <fgColor rgb="FFCC0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCC0000"/>
+        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -89,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -112,6 +112,50 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -130,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -228,33 +272,20 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -622,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S242"/>
+  <dimension ref="A1:S241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2948,52 +2979,52 @@
       <c r="S40" s="14" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="32" t="inlineStr">
+      <c r="A41" s="26" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="B41" s="32" t="n"/>
-      <c r="C41" s="33" t="inlineStr">
+      <c r="B41" s="26" t="n"/>
+      <c r="C41" s="27" t="inlineStr">
         <is>
           <t>Chili</t>
         </is>
       </c>
-      <c r="D41" s="33" t="n"/>
-      <c r="E41" s="32" t="n"/>
-      <c r="F41" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="34" t="n">
+      <c r="D41" s="27" t="n"/>
+      <c r="E41" s="26" t="n"/>
+      <c r="F41" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="28" t="n">
         <v>17.8</v>
       </c>
-      <c r="H41" s="35" t="n">
+      <c r="H41" s="29" t="n">
         <v>17.8</v>
       </c>
-      <c r="I41" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" s="35" t="n">
+      <c r="I41" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="29" t="n">
         <v>17.8</v>
       </c>
-      <c r="L41" s="33" t="inlineStr">
+      <c r="L41" s="27" t="inlineStr">
         <is>
           <t>per Sleeve (None)</t>
         </is>
       </c>
-      <c r="M41" s="32" t="n"/>
-      <c r="N41" s="34">
+      <c r="M41" s="26" t="n"/>
+      <c r="N41" s="28">
         <f>M41*G41</f>
         <v/>
       </c>
-      <c r="O41" s="32" t="n"/>
-      <c r="P41" s="32" t="n"/>
-      <c r="Q41" s="32" t="n"/>
-      <c r="R41" s="32" t="n"/>
-      <c r="S41" s="32" t="n"/>
+      <c r="O41" s="26" t="n"/>
+      <c r="P41" s="26" t="n"/>
+      <c r="Q41" s="26" t="n"/>
+      <c r="R41" s="26" t="n"/>
+      <c r="S41" s="26" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -4514,52 +4545,52 @@
       <c r="S68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="32" t="inlineStr">
+      <c r="A69" s="26" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B69" s="32" t="n"/>
-      <c r="C69" s="33" t="inlineStr">
+      <c r="B69" s="26" t="n"/>
+      <c r="C69" s="27" t="inlineStr">
         <is>
           <t>Donut Apple</t>
         </is>
       </c>
-      <c r="D69" s="33" t="n"/>
-      <c r="E69" s="32" t="n"/>
-      <c r="F69" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" s="34" t="n">
+      <c r="D69" s="27" t="n"/>
+      <c r="E69" s="26" t="n"/>
+      <c r="F69" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="28" t="n">
         <v>33.26</v>
       </c>
-      <c r="H69" s="35" t="n">
+      <c r="H69" s="29" t="n">
         <v>33.26</v>
       </c>
-      <c r="I69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" s="35" t="n">
+      <c r="I69" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="29" t="n">
         <v>33.26</v>
       </c>
-      <c r="L69" s="33" t="inlineStr">
+      <c r="L69" s="27" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M69" s="32" t="n"/>
-      <c r="N69" s="34">
+      <c r="M69" s="26" t="n"/>
+      <c r="N69" s="28">
         <f>M69*G69</f>
         <v/>
       </c>
-      <c r="O69" s="32" t="n"/>
-      <c r="P69" s="32" t="n"/>
-      <c r="Q69" s="32" t="n"/>
-      <c r="R69" s="32" t="n"/>
-      <c r="S69" s="32" t="n"/>
+      <c r="O69" s="26" t="n"/>
+      <c r="P69" s="26" t="n"/>
+      <c r="Q69" s="26" t="n"/>
+      <c r="R69" s="26" t="n"/>
+      <c r="S69" s="26" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -10604,52 +10635,52 @@
       <c r="S174" s="8" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="32" t="inlineStr">
+      <c r="A175" s="26" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="B175" s="32" t="n"/>
-      <c r="C175" s="33" t="inlineStr">
+      <c r="B175" s="26" t="n"/>
+      <c r="C175" s="27" t="inlineStr">
         <is>
           <t>Soup Cream of Mushroom</t>
         </is>
       </c>
-      <c r="D175" s="33" t="n"/>
-      <c r="E175" s="32" t="n"/>
-      <c r="F175" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G175" s="34" t="n">
+      <c r="D175" s="27" t="n"/>
+      <c r="E175" s="26" t="n"/>
+      <c r="F175" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G175" s="28" t="n">
         <v>5.79</v>
       </c>
-      <c r="H175" s="35" t="n">
+      <c r="H175" s="29" t="n">
         <v>5.79</v>
       </c>
-      <c r="I175" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J175" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K175" s="35" t="n">
+      <c r="I175" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K175" s="29" t="n">
         <v>5.79</v>
       </c>
-      <c r="L175" s="33" t="inlineStr">
+      <c r="L175" s="27" t="inlineStr">
         <is>
           <t>per Can (None)</t>
         </is>
       </c>
-      <c r="M175" s="32" t="n"/>
-      <c r="N175" s="34">
+      <c r="M175" s="26" t="n"/>
+      <c r="N175" s="28">
         <f>M175*G175</f>
         <v/>
       </c>
-      <c r="O175" s="32" t="n"/>
-      <c r="P175" s="32" t="n"/>
-      <c r="Q175" s="32" t="n"/>
-      <c r="R175" s="32" t="n"/>
-      <c r="S175" s="32" t="n"/>
+      <c r="O175" s="26" t="n"/>
+      <c r="P175" s="26" t="n"/>
+      <c r="Q175" s="26" t="n"/>
+      <c r="R175" s="26" t="n"/>
+      <c r="S175" s="26" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -11848,1953 +11879,1939 @@
       <c r="S196" s="20" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="32" t="inlineStr">
+      <c r="A197" s="26" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B197" s="32" t="n"/>
-      <c r="C197" s="33" t="inlineStr">
+      <c r="B197" s="26" t="n"/>
+      <c r="C197" s="27" t="inlineStr">
         <is>
           <t>Lettuce Head</t>
         </is>
       </c>
-      <c r="D197" s="33" t="n"/>
-      <c r="E197" s="32" t="n"/>
-      <c r="F197" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G197" s="34" t="n">
+      <c r="D197" s="27" t="n"/>
+      <c r="E197" s="26" t="n"/>
+      <c r="F197" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G197" s="28" t="n">
         <v>3.99</v>
       </c>
-      <c r="H197" s="35" t="n">
+      <c r="H197" s="29" t="n">
         <v>3.99</v>
       </c>
-      <c r="I197" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J197" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K197" s="35" t="n">
+      <c r="I197" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J197" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K197" s="29" t="n">
         <v>3.99</v>
       </c>
-      <c r="L197" s="33" t="inlineStr">
+      <c r="L197" s="27" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M197" s="32" t="n"/>
-      <c r="N197" s="34">
+      <c r="M197" s="26" t="n"/>
+      <c r="N197" s="28">
         <f>M197*G197</f>
         <v/>
       </c>
-      <c r="O197" s="32" t="n"/>
-      <c r="P197" s="32" t="n"/>
-      <c r="Q197" s="32" t="n"/>
-      <c r="R197" s="32" t="n"/>
-      <c r="S197" s="32" t="n"/>
+      <c r="O197" s="26" t="n"/>
+      <c r="P197" s="26" t="n"/>
+      <c r="Q197" s="26" t="n"/>
+      <c r="R197" s="26" t="n"/>
+      <c r="S197" s="26" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="32" t="inlineStr">
+      <c r="A198" s="26" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B198" s="32" t="n"/>
-      <c r="C198" s="33" t="inlineStr">
+      <c r="B198" s="26" t="n"/>
+      <c r="C198" s="27" t="inlineStr">
         <is>
           <t>Tomato</t>
         </is>
       </c>
-      <c r="D198" s="33" t="n"/>
-      <c r="E198" s="32" t="n"/>
-      <c r="F198" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G198" s="34" t="n">
+      <c r="D198" s="27" t="n"/>
+      <c r="E198" s="26" t="n"/>
+      <c r="F198" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G198" s="28" t="n">
         <v>2.49</v>
       </c>
-      <c r="H198" s="35" t="n">
+      <c r="H198" s="29" t="n">
         <v>2.49</v>
       </c>
-      <c r="I198" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J198" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K198" s="35" t="n">
+      <c r="I198" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J198" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K198" s="29" t="n">
         <v>2.49</v>
       </c>
-      <c r="L198" s="33" t="inlineStr">
+      <c r="L198" s="27" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M198" s="32" t="n"/>
-      <c r="N198" s="34">
+      <c r="M198" s="26" t="n"/>
+      <c r="N198" s="28">
         <f>M198*G198</f>
         <v/>
       </c>
-      <c r="O198" s="32" t="n"/>
-      <c r="P198" s="32" t="n"/>
-      <c r="Q198" s="32" t="n"/>
-      <c r="R198" s="32" t="n"/>
-      <c r="S198" s="32" t="n"/>
+      <c r="O198" s="26" t="n"/>
+      <c r="P198" s="26" t="n"/>
+      <c r="Q198" s="26" t="n"/>
+      <c r="R198" s="26" t="n"/>
+      <c r="S198" s="26" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="32" t="inlineStr">
+      <c r="A199" s="26" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B199" s="32" t="n"/>
-      <c r="C199" s="33" t="inlineStr">
+      <c r="B199" s="26" t="n"/>
+      <c r="C199" s="27" t="inlineStr">
         <is>
           <t>Creole Marinade</t>
         </is>
       </c>
-      <c r="D199" s="33" t="n"/>
-      <c r="E199" s="32" t="n"/>
-      <c r="F199" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G199" s="34" t="n">
+      <c r="D199" s="27" t="n"/>
+      <c r="E199" s="26" t="n"/>
+      <c r="F199" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G199" s="28" t="n">
         <v>1.81</v>
       </c>
-      <c r="H199" s="35" t="n">
+      <c r="H199" s="29" t="n">
         <v>1.81</v>
       </c>
-      <c r="I199" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J199" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K199" s="35" t="n">
+      <c r="I199" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J199" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K199" s="29" t="n">
         <v>1.81</v>
       </c>
-      <c r="L199" s="33" t="inlineStr">
+      <c r="L199" s="27" t="inlineStr">
         <is>
           <t>per Bag (None)</t>
         </is>
       </c>
-      <c r="M199" s="32" t="n"/>
-      <c r="N199" s="34">
+      <c r="M199" s="26" t="n"/>
+      <c r="N199" s="28">
         <f>M199*G199</f>
         <v/>
       </c>
-      <c r="O199" s="32" t="n"/>
-      <c r="P199" s="32" t="n"/>
-      <c r="Q199" s="32" t="n"/>
-      <c r="R199" s="32" t="n"/>
-      <c r="S199" s="32" t="n"/>
+      <c r="O199" s="26" t="n"/>
+      <c r="P199" s="26" t="n"/>
+      <c r="Q199" s="26" t="n"/>
+      <c r="R199" s="26" t="n"/>
+      <c r="S199" s="26" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="32" t="inlineStr">
+      <c r="A200" s="26" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B200" s="32" t="n"/>
-      <c r="C200" s="33" t="inlineStr">
+      <c r="B200" s="26" t="n"/>
+      <c r="C200" s="27" t="inlineStr">
         <is>
           <t>Spicy Marinade</t>
         </is>
       </c>
-      <c r="D200" s="33" t="n"/>
-      <c r="E200" s="32" t="n"/>
-      <c r="F200" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G200" s="34" t="n">
+      <c r="D200" s="27" t="n"/>
+      <c r="E200" s="26" t="n"/>
+      <c r="F200" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G200" s="28" t="n">
         <v>5.27</v>
       </c>
-      <c r="H200" s="35" t="n">
+      <c r="H200" s="29" t="n">
         <v>5.27</v>
       </c>
-      <c r="I200" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J200" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K200" s="35" t="n">
+      <c r="I200" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J200" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K200" s="29" t="n">
         <v>5.27</v>
       </c>
-      <c r="L200" s="33" t="inlineStr">
+      <c r="L200" s="27" t="inlineStr">
         <is>
           <t>per Bag (None)</t>
         </is>
       </c>
-      <c r="M200" s="32" t="n"/>
-      <c r="N200" s="34">
+      <c r="M200" s="26" t="n"/>
+      <c r="N200" s="28">
         <f>M200*G200</f>
         <v/>
       </c>
-      <c r="O200" s="32" t="n"/>
-      <c r="P200" s="32" t="n"/>
-      <c r="Q200" s="32" t="n"/>
-      <c r="R200" s="32" t="n"/>
-      <c r="S200" s="32" t="n"/>
+      <c r="O200" s="26" t="n"/>
+      <c r="P200" s="26" t="n"/>
+      <c r="Q200" s="26" t="n"/>
+      <c r="R200" s="26" t="n"/>
+      <c r="S200" s="26" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="32" t="inlineStr">
+      <c r="A201" s="26" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B201" s="32" t="n"/>
-      <c r="C201" s="33" t="inlineStr">
+      <c r="B201" s="26" t="n"/>
+      <c r="C201" s="27" t="inlineStr">
         <is>
           <t>Batter Mix</t>
         </is>
       </c>
-      <c r="D201" s="33" t="n"/>
-      <c r="E201" s="32" t="n"/>
-      <c r="F201" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G201" s="34" t="n">
+      <c r="D201" s="27" t="n"/>
+      <c r="E201" s="26" t="n"/>
+      <c r="F201" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G201" s="28" t="n">
         <v>2.5</v>
       </c>
-      <c r="H201" s="35" t="n">
+      <c r="H201" s="29" t="n">
         <v>2.5</v>
       </c>
-      <c r="I201" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J201" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K201" s="35" t="n">
+      <c r="I201" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J201" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K201" s="29" t="n">
         <v>2.5</v>
       </c>
-      <c r="L201" s="33" t="inlineStr">
+      <c r="L201" s="27" t="inlineStr">
         <is>
           <t>per Bag (None)</t>
         </is>
       </c>
-      <c r="M201" s="32" t="n"/>
-      <c r="N201" s="34">
+      <c r="M201" s="26" t="n"/>
+      <c r="N201" s="28">
         <f>M201*G201</f>
         <v/>
       </c>
-      <c r="O201" s="32" t="n"/>
-      <c r="P201" s="32" t="n"/>
-      <c r="Q201" s="32" t="n"/>
-      <c r="R201" s="32" t="n"/>
-      <c r="S201" s="32" t="n"/>
-    </row>
-    <row r="202">
-      <c r="A202" s="26" t="n"/>
-      <c r="B202" s="26" t="inlineStr">
-        <is>
-          <t>Imperial</t>
-        </is>
-      </c>
-      <c r="C202" s="27" t="n"/>
-      <c r="D202" s="27" t="n"/>
-      <c r="E202" s="26" t="n"/>
-      <c r="F202" s="26" t="n"/>
-      <c r="G202" s="28" t="n"/>
-      <c r="H202" s="29" t="n"/>
-      <c r="I202" s="30" t="n"/>
-      <c r="J202" s="31" t="n"/>
-      <c r="K202" s="29" t="n"/>
-      <c r="L202" s="27" t="inlineStr">
-        <is>
-          <t>see label</t>
-        </is>
-      </c>
-      <c r="M202" s="26" t="n"/>
-      <c r="N202" s="28">
-        <f>M202*G202</f>
-        <v/>
-      </c>
-      <c r="O202" s="26" t="n"/>
-      <c r="P202" s="26" t="n"/>
-      <c r="Q202" s="26" t="n"/>
-      <c r="R202" s="26" t="n"/>
-      <c r="S202" s="26" t="n"/>
+      <c r="O201" s="26" t="n"/>
+      <c r="P201" s="26" t="n"/>
+      <c r="Q201" s="26" t="n"/>
+      <c r="R201" s="26" t="n"/>
+      <c r="S201" s="26" t="n"/>
+    </row>
+    <row r="202" ht="18" customHeight="1">
+      <c r="A202" s="32" t="inlineStr">
+        <is>
+          <t>─── IMPERIAL / LOCAL VENDORS (prices not in BEK) ───</t>
+        </is>
+      </c>
+      <c r="B202" s="33" t="n"/>
+      <c r="C202" s="33" t="n"/>
+      <c r="D202" s="33" t="n"/>
+      <c r="E202" s="33" t="n"/>
+      <c r="F202" s="33" t="n"/>
+      <c r="G202" s="33" t="n"/>
+      <c r="H202" s="33" t="n"/>
+      <c r="I202" s="33" t="n"/>
+      <c r="J202" s="33" t="n"/>
+      <c r="K202" s="33" t="n"/>
+      <c r="L202" s="33" t="n"/>
+      <c r="M202" s="33" t="n"/>
+      <c r="N202" s="33" t="n"/>
+      <c r="O202" s="33" t="n"/>
+      <c r="P202" s="33" t="n"/>
+      <c r="Q202" s="33" t="n"/>
+      <c r="R202" s="33" t="n"/>
+      <c r="S202" s="34" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="32" t="inlineStr">
+      <c r="A203" s="2" t="inlineStr">
         <is>
           <t>PACK</t>
         </is>
       </c>
-      <c r="B203" s="32" t="n"/>
-      <c r="C203" s="33" t="inlineStr">
+      <c r="B203" s="2" t="n"/>
+      <c r="C203" s="3" t="inlineStr">
         <is>
           <t>Bayou Blend Pork</t>
         </is>
       </c>
-      <c r="D203" s="33" t="n"/>
-      <c r="E203" s="32" t="inlineStr">
+      <c r="D203" s="3" t="n"/>
+      <c r="E203" s="2" t="inlineStr">
         <is>
           <t>5 Packs</t>
         </is>
       </c>
-      <c r="F203" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G203" s="34" t="n">
+      <c r="F203" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G203" s="4" t="n">
         <v>7.48</v>
       </c>
-      <c r="H203" s="35" t="n">
+      <c r="H203" s="5" t="n">
         <v>7.48</v>
       </c>
-      <c r="I203" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J203" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K203" s="35" t="n">
+      <c r="I203" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J203" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K203" s="5" t="n">
         <v>1.496</v>
       </c>
-      <c r="L203" s="33" t="inlineStr">
+      <c r="L203" s="3" t="inlineStr">
         <is>
           <t>per Pack (5 Packs)</t>
         </is>
       </c>
-      <c r="M203" s="32" t="n"/>
-      <c r="N203" s="34">
+      <c r="M203" s="2" t="n"/>
+      <c r="N203" s="4">
         <f>M203*G203</f>
         <v/>
       </c>
-      <c r="O203" s="32" t="n"/>
-      <c r="P203" s="32" t="n"/>
-      <c r="Q203" s="32" t="n"/>
-      <c r="R203" s="32" t="n"/>
-      <c r="S203" s="32" t="n"/>
+      <c r="O203" s="2" t="n"/>
+      <c r="P203" s="2" t="n"/>
+      <c r="Q203" s="2" t="n"/>
+      <c r="R203" s="2" t="n"/>
+      <c r="S203" s="2" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="32" t="inlineStr">
+      <c r="A204" s="2" t="inlineStr">
         <is>
           <t>PACK</t>
         </is>
       </c>
-      <c r="B204" s="32" t="n"/>
-      <c r="C204" s="33" t="inlineStr">
+      <c r="B204" s="2" t="n"/>
+      <c r="C204" s="3" t="inlineStr">
         <is>
           <t>Bayou Blend Alligator</t>
         </is>
       </c>
-      <c r="D204" s="33" t="n"/>
-      <c r="E204" s="32" t="inlineStr">
+      <c r="D204" s="3" t="n"/>
+      <c r="E204" s="2" t="inlineStr">
         <is>
           <t>5 Pack</t>
         </is>
       </c>
-      <c r="F204" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G204" s="34" t="n">
+      <c r="F204" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G204" s="4" t="n">
         <v>9.890000000000001</v>
       </c>
-      <c r="H204" s="35" t="n">
+      <c r="H204" s="5" t="n">
         <v>9.890000000000001</v>
       </c>
-      <c r="I204" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J204" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K204" s="35" t="n">
+      <c r="I204" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J204" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K204" s="5" t="n">
         <v>1.978</v>
       </c>
-      <c r="L204" s="33" t="inlineStr">
+      <c r="L204" s="3" t="inlineStr">
         <is>
           <t>per Pack (5 Pack)</t>
         </is>
       </c>
-      <c r="M204" s="32" t="n"/>
-      <c r="N204" s="34">
+      <c r="M204" s="2" t="n"/>
+      <c r="N204" s="4">
         <f>M204*G204</f>
         <v/>
       </c>
-      <c r="O204" s="32" t="n"/>
-      <c r="P204" s="32" t="n"/>
-      <c r="Q204" s="32" t="n"/>
-      <c r="R204" s="32" t="n"/>
-      <c r="S204" s="32" t="n"/>
+      <c r="O204" s="2" t="n"/>
+      <c r="P204" s="2" t="n"/>
+      <c r="Q204" s="2" t="n"/>
+      <c r="R204" s="2" t="n"/>
+      <c r="S204" s="2" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" s="32" t="inlineStr">
+      <c r="A205" s="2" t="inlineStr">
         <is>
           <t>PACK</t>
         </is>
       </c>
-      <c r="B205" s="32" t="n"/>
-      <c r="C205" s="33" t="inlineStr">
+      <c r="B205" s="2" t="n"/>
+      <c r="C205" s="3" t="inlineStr">
         <is>
           <t>Bayou Blend Crawfish</t>
         </is>
       </c>
-      <c r="D205" s="33" t="n"/>
-      <c r="E205" s="32" t="inlineStr">
+      <c r="D205" s="3" t="n"/>
+      <c r="E205" s="2" t="inlineStr">
         <is>
           <t>5 Packs</t>
         </is>
       </c>
-      <c r="F205" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G205" s="34" t="n">
+      <c r="F205" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G205" s="4" t="n">
         <v>9.1</v>
       </c>
-      <c r="H205" s="35" t="n">
+      <c r="H205" s="5" t="n">
         <v>9.1</v>
       </c>
-      <c r="I205" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J205" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K205" s="35" t="n">
+      <c r="I205" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J205" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K205" s="5" t="n">
         <v>1.82</v>
       </c>
-      <c r="L205" s="33" t="inlineStr">
+      <c r="L205" s="3" t="inlineStr">
         <is>
           <t>per Pack (5 Packs)</t>
         </is>
       </c>
-      <c r="M205" s="32" t="n"/>
-      <c r="N205" s="34">
+      <c r="M205" s="2" t="n"/>
+      <c r="N205" s="4">
         <f>M205*G205</f>
         <v/>
       </c>
-      <c r="O205" s="32" t="n"/>
-      <c r="P205" s="32" t="n"/>
-      <c r="Q205" s="32" t="n"/>
-      <c r="R205" s="32" t="n"/>
-      <c r="S205" s="32" t="n"/>
+      <c r="O205" s="2" t="n"/>
+      <c r="P205" s="2" t="n"/>
+      <c r="Q205" s="2" t="n"/>
+      <c r="R205" s="2" t="n"/>
+      <c r="S205" s="2" t="n"/>
     </row>
     <row r="206">
-      <c r="A206" s="32" t="inlineStr">
+      <c r="A206" s="2" t="inlineStr">
         <is>
           <t>PACK</t>
         </is>
       </c>
-      <c r="B206" s="32" t="n"/>
-      <c r="C206" s="33" t="inlineStr">
+      <c r="B206" s="2" t="n"/>
+      <c r="C206" s="3" t="inlineStr">
         <is>
           <t>Bayou Blend Shrimp</t>
         </is>
       </c>
-      <c r="D206" s="33" t="n"/>
-      <c r="E206" s="32" t="inlineStr">
+      <c r="D206" s="3" t="n"/>
+      <c r="E206" s="2" t="inlineStr">
         <is>
           <t>5 Packs</t>
         </is>
       </c>
-      <c r="F206" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G206" s="34" t="n">
+      <c r="F206" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G206" s="4" t="n">
         <v>8.08</v>
       </c>
-      <c r="H206" s="35" t="n">
+      <c r="H206" s="5" t="n">
         <v>8.08</v>
       </c>
-      <c r="I206" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J206" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K206" s="35" t="n">
+      <c r="I206" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J206" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K206" s="5" t="n">
         <v>1.616</v>
       </c>
-      <c r="L206" s="33" t="inlineStr">
+      <c r="L206" s="3" t="inlineStr">
         <is>
           <t>per Pack (5 Packs)</t>
         </is>
       </c>
-      <c r="M206" s="32" t="n"/>
-      <c r="N206" s="34">
+      <c r="M206" s="2" t="n"/>
+      <c r="N206" s="4">
         <f>M206*G206</f>
         <v/>
       </c>
-      <c r="O206" s="32" t="n"/>
-      <c r="P206" s="32" t="n"/>
-      <c r="Q206" s="32" t="n"/>
-      <c r="R206" s="32" t="n"/>
-      <c r="S206" s="32" t="n"/>
+      <c r="O206" s="2" t="n"/>
+      <c r="P206" s="2" t="n"/>
+      <c r="Q206" s="2" t="n"/>
+      <c r="R206" s="2" t="n"/>
+      <c r="S206" s="2" t="n"/>
     </row>
     <row r="207">
-      <c r="A207" s="32" t="inlineStr">
+      <c r="A207" s="2" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="B207" s="32" t="n"/>
-      <c r="C207" s="33" t="inlineStr">
+      <c r="B207" s="2" t="n"/>
+      <c r="C207" s="3" t="inlineStr">
         <is>
           <t>Peanuts Regular/Cajun</t>
         </is>
       </c>
-      <c r="D207" s="33" t="n"/>
-      <c r="E207" s="32" t="inlineStr">
+      <c r="D207" s="3" t="n"/>
+      <c r="E207" s="2" t="inlineStr">
         <is>
           <t>6 Cans</t>
         </is>
       </c>
-      <c r="F207" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G207" s="34" t="n">
+      <c r="F207" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G207" s="4" t="n">
         <v>8.33</v>
       </c>
-      <c r="H207" s="35" t="n">
+      <c r="H207" s="5" t="n">
         <v>8.33</v>
       </c>
-      <c r="I207" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J207" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K207" s="35" t="n">
+      <c r="I207" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J207" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K207" s="5" t="n">
         <v>1.388333333333333</v>
       </c>
-      <c r="L207" s="33" t="inlineStr">
+      <c r="L207" s="3" t="inlineStr">
         <is>
           <t>per Can (6 Cans)</t>
         </is>
       </c>
-      <c r="M207" s="32" t="n"/>
-      <c r="N207" s="34">
+      <c r="M207" s="2" t="n"/>
+      <c r="N207" s="4">
         <f>M207*G207</f>
         <v/>
       </c>
-      <c r="O207" s="32" t="n"/>
-      <c r="P207" s="32" t="n"/>
-      <c r="Q207" s="32" t="n"/>
-      <c r="R207" s="32" t="n"/>
-      <c r="S207" s="32" t="n"/>
+      <c r="O207" s="2" t="n"/>
+      <c r="P207" s="2" t="n"/>
+      <c r="Q207" s="2" t="n"/>
+      <c r="R207" s="2" t="n"/>
+      <c r="S207" s="2" t="n"/>
     </row>
     <row r="208">
-      <c r="A208" s="32" t="inlineStr">
+      <c r="A208" s="2" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="B208" s="32" t="n"/>
-      <c r="C208" s="33" t="inlineStr">
+      <c r="B208" s="2" t="n"/>
+      <c r="C208" s="3" t="inlineStr">
         <is>
           <t>16oz Peanut Cup</t>
         </is>
       </c>
-      <c r="D208" s="33" t="n"/>
-      <c r="E208" s="32" t="inlineStr">
+      <c r="D208" s="3" t="n"/>
+      <c r="E208" s="2" t="inlineStr">
         <is>
           <t>20 Sleeves</t>
         </is>
       </c>
-      <c r="F208" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G208" s="34" t="n">
+      <c r="F208" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G208" s="4" t="n">
         <v>8.01</v>
       </c>
-      <c r="H208" s="35" t="n">
+      <c r="H208" s="5" t="n">
         <v>8.01</v>
       </c>
-      <c r="I208" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J208" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K208" s="35" t="n">
+      <c r="I208" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J208" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K208" s="5" t="n">
         <v>0.4005</v>
       </c>
-      <c r="L208" s="33" t="inlineStr">
+      <c r="L208" s="3" t="inlineStr">
         <is>
           <t>per Sleeve (20 Sleeves)</t>
         </is>
       </c>
-      <c r="M208" s="32" t="n"/>
-      <c r="N208" s="34">
+      <c r="M208" s="2" t="n"/>
+      <c r="N208" s="4">
         <f>M208*G208</f>
         <v/>
       </c>
-      <c r="O208" s="32" t="n"/>
-      <c r="P208" s="32" t="n"/>
-      <c r="Q208" s="32" t="n"/>
-      <c r="R208" s="32" t="n"/>
-      <c r="S208" s="32" t="n"/>
+      <c r="O208" s="2" t="n"/>
+      <c r="P208" s="2" t="n"/>
+      <c r="Q208" s="2" t="n"/>
+      <c r="R208" s="2" t="n"/>
+      <c r="S208" s="2" t="n"/>
     </row>
     <row r="209">
-      <c r="A209" s="32" t="inlineStr">
+      <c r="A209" s="2" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="B209" s="32" t="n"/>
-      <c r="C209" s="33" t="inlineStr">
+      <c r="B209" s="2" t="n"/>
+      <c r="C209" s="3" t="inlineStr">
         <is>
           <t>32oz Peanut Cup</t>
         </is>
       </c>
-      <c r="D209" s="33" t="n"/>
-      <c r="E209" s="32" t="inlineStr">
+      <c r="D209" s="3" t="n"/>
+      <c r="E209" s="2" t="inlineStr">
         <is>
           <t>20 Sleeves</t>
         </is>
       </c>
-      <c r="F209" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G209" s="34" t="n">
+      <c r="F209" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G209" s="4" t="n">
         <v>10.22</v>
       </c>
-      <c r="H209" s="35" t="n">
+      <c r="H209" s="5" t="n">
         <v>10.22</v>
       </c>
-      <c r="I209" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J209" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K209" s="35" t="n">
+      <c r="I209" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J209" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K209" s="5" t="n">
         <v>0.511</v>
       </c>
-      <c r="L209" s="33" t="inlineStr">
+      <c r="L209" s="3" t="inlineStr">
         <is>
           <t>per Sleeve (20 Sleeves)</t>
         </is>
       </c>
-      <c r="M209" s="32" t="n"/>
-      <c r="N209" s="34">
+      <c r="M209" s="2" t="n"/>
+      <c r="N209" s="4">
         <f>M209*G209</f>
         <v/>
       </c>
-      <c r="O209" s="32" t="n"/>
-      <c r="P209" s="32" t="n"/>
-      <c r="Q209" s="32" t="n"/>
-      <c r="R209" s="32" t="n"/>
-      <c r="S209" s="32" t="n"/>
+      <c r="O209" s="2" t="n"/>
+      <c r="P209" s="2" t="n"/>
+      <c r="Q209" s="2" t="n"/>
+      <c r="R209" s="2" t="n"/>
+      <c r="S209" s="2" t="n"/>
     </row>
     <row r="210">
-      <c r="A210" s="32" t="inlineStr">
+      <c r="A210" s="2" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="B210" s="32" t="n"/>
-      <c r="C210" s="33" t="inlineStr">
+      <c r="B210" s="2" t="n"/>
+      <c r="C210" s="3" t="inlineStr">
         <is>
           <t>Peanut Cup Lid</t>
         </is>
       </c>
-      <c r="D210" s="33" t="n"/>
-      <c r="E210" s="32" t="inlineStr">
+      <c r="D210" s="3" t="n"/>
+      <c r="E210" s="2" t="inlineStr">
         <is>
           <t>10 Sleeves</t>
         </is>
       </c>
-      <c r="F210" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G210" s="34" t="n">
+      <c r="F210" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G210" s="4" t="n">
         <v>5.01</v>
       </c>
-      <c r="H210" s="35" t="n">
+      <c r="H210" s="5" t="n">
         <v>5.01</v>
       </c>
-      <c r="I210" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J210" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K210" s="35" t="n">
+      <c r="I210" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K210" s="5" t="n">
         <v>0.501</v>
       </c>
-      <c r="L210" s="33" t="inlineStr">
+      <c r="L210" s="3" t="inlineStr">
         <is>
           <t>per Sleeve (10 Sleeves)</t>
         </is>
       </c>
-      <c r="M210" s="32" t="n"/>
-      <c r="N210" s="34">
+      <c r="M210" s="2" t="n"/>
+      <c r="N210" s="4">
         <f>M210*G210</f>
         <v/>
       </c>
-      <c r="O210" s="32" t="n"/>
-      <c r="P210" s="32" t="n"/>
-      <c r="Q210" s="32" t="n"/>
-      <c r="R210" s="32" t="n"/>
-      <c r="S210" s="32" t="n"/>
+      <c r="O210" s="2" t="n"/>
+      <c r="P210" s="2" t="n"/>
+      <c r="Q210" s="2" t="n"/>
+      <c r="R210" s="2" t="n"/>
+      <c r="S210" s="2" t="n"/>
     </row>
     <row r="211">
-      <c r="A211" s="32" t="inlineStr">
+      <c r="A211" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B211" s="32" t="n"/>
-      <c r="C211" s="33" t="inlineStr">
+      <c r="B211" s="2" t="n"/>
+      <c r="C211" s="3" t="inlineStr">
         <is>
           <t>Gizzards</t>
         </is>
       </c>
-      <c r="D211" s="33" t="n"/>
-      <c r="E211" s="32" t="inlineStr">
+      <c r="D211" s="3" t="n"/>
+      <c r="E211" s="2" t="inlineStr">
         <is>
           <t>4/Box</t>
         </is>
       </c>
-      <c r="F211" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G211" s="34" t="n">
+      <c r="F211" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G211" s="4" t="n">
         <v>19.8</v>
       </c>
-      <c r="H211" s="35" t="n">
+      <c r="H211" s="5" t="n">
         <v>19.8</v>
       </c>
-      <c r="I211" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J211" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K211" s="35" t="n">
+      <c r="I211" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K211" s="5" t="n">
         <v>4.95</v>
       </c>
-      <c r="L211" s="33" t="inlineStr">
+      <c r="L211" s="3" t="inlineStr">
         <is>
           <t>per Bag (4/Box)</t>
         </is>
       </c>
-      <c r="M211" s="32" t="n"/>
-      <c r="N211" s="34">
+      <c r="M211" s="2" t="n"/>
+      <c r="N211" s="4">
         <f>M211*G211</f>
         <v/>
       </c>
-      <c r="O211" s="32" t="n"/>
-      <c r="P211" s="32" t="n"/>
-      <c r="Q211" s="32" t="n"/>
-      <c r="R211" s="32" t="n"/>
-      <c r="S211" s="32" t="n"/>
+      <c r="O211" s="2" t="n"/>
+      <c r="P211" s="2" t="n"/>
+      <c r="Q211" s="2" t="n"/>
+      <c r="R211" s="2" t="n"/>
+      <c r="S211" s="2" t="n"/>
     </row>
     <row r="212">
-      <c r="A212" s="32" t="inlineStr">
+      <c r="A212" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B212" s="32" t="n"/>
-      <c r="C212" s="33" t="inlineStr">
+      <c r="B212" s="2" t="n"/>
+      <c r="C212" s="3" t="inlineStr">
         <is>
           <t>Livers</t>
         </is>
       </c>
-      <c r="D212" s="33" t="n"/>
-      <c r="E212" s="32" t="inlineStr">
+      <c r="D212" s="3" t="n"/>
+      <c r="E212" s="2" t="inlineStr">
         <is>
           <t>4/Box</t>
         </is>
       </c>
-      <c r="F212" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G212" s="34" t="n">
+      <c r="F212" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G212" s="4" t="n">
         <v>14.78</v>
       </c>
-      <c r="H212" s="35" t="n">
+      <c r="H212" s="5" t="n">
         <v>14.78</v>
       </c>
-      <c r="I212" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J212" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K212" s="35" t="n">
+      <c r="I212" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J212" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K212" s="5" t="n">
         <v>3.695</v>
       </c>
-      <c r="L212" s="33" t="inlineStr">
+      <c r="L212" s="3" t="inlineStr">
         <is>
           <t>per Bag (4/Box)</t>
         </is>
       </c>
-      <c r="M212" s="32" t="n"/>
-      <c r="N212" s="34">
+      <c r="M212" s="2" t="n"/>
+      <c r="N212" s="4">
         <f>M212*G212</f>
         <v/>
       </c>
-      <c r="O212" s="32" t="n"/>
-      <c r="P212" s="32" t="n"/>
-      <c r="Q212" s="32" t="n"/>
-      <c r="R212" s="32" t="n"/>
-      <c r="S212" s="32" t="n"/>
+      <c r="O212" s="2" t="n"/>
+      <c r="P212" s="2" t="n"/>
+      <c r="Q212" s="2" t="n"/>
+      <c r="R212" s="2" t="n"/>
+      <c r="S212" s="2" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" s="32" t="inlineStr">
+      <c r="A213" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B213" s="32" t="n"/>
-      <c r="C213" s="33" t="inlineStr">
+      <c r="B213" s="2" t="n"/>
+      <c r="C213" s="3" t="inlineStr">
         <is>
           <t>Brisket</t>
         </is>
       </c>
-      <c r="D213" s="33" t="n"/>
-      <c r="E213" s="32" t="n"/>
-      <c r="F213" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G213" s="34" t="n">
+      <c r="D213" s="3" t="n"/>
+      <c r="E213" s="2" t="n"/>
+      <c r="F213" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G213" s="4" t="n">
         <v>29.44</v>
       </c>
-      <c r="H213" s="35" t="n">
+      <c r="H213" s="5" t="n">
         <v>29.44</v>
       </c>
-      <c r="I213" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J213" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K213" s="35" t="n">
+      <c r="I213" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J213" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K213" s="5" t="n">
         <v>29.44</v>
       </c>
-      <c r="L213" s="33" t="inlineStr">
+      <c r="L213" s="3" t="inlineStr">
         <is>
           <t>per Bag (None)</t>
         </is>
       </c>
-      <c r="M213" s="32" t="n"/>
-      <c r="N213" s="34">
+      <c r="M213" s="2" t="n"/>
+      <c r="N213" s="4">
         <f>M213*G213</f>
         <v/>
       </c>
-      <c r="O213" s="32" t="n"/>
-      <c r="P213" s="32" t="n"/>
-      <c r="Q213" s="32" t="n"/>
-      <c r="R213" s="32" t="n"/>
-      <c r="S213" s="32" t="n"/>
+      <c r="O213" s="2" t="n"/>
+      <c r="P213" s="2" t="n"/>
+      <c r="Q213" s="2" t="n"/>
+      <c r="R213" s="2" t="n"/>
+      <c r="S213" s="2" t="n"/>
     </row>
     <row r="214">
-      <c r="A214" s="32" t="inlineStr">
+      <c r="A214" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B214" s="32" t="n"/>
-      <c r="C214" s="33" t="inlineStr">
+      <c r="B214" s="2" t="n"/>
+      <c r="C214" s="3" t="inlineStr">
         <is>
           <t>Kolache Boudin Link Org</t>
         </is>
       </c>
-      <c r="D214" s="33" t="n"/>
-      <c r="E214" s="32" t="n"/>
-      <c r="F214" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G214" s="34" t="n">
+      <c r="D214" s="3" t="n"/>
+      <c r="E214" s="2" t="n"/>
+      <c r="F214" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G214" s="4" t="n">
         <v>69.77</v>
       </c>
-      <c r="H214" s="35" t="n">
+      <c r="H214" s="5" t="n">
         <v>69.77</v>
       </c>
-      <c r="I214" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J214" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K214" s="35" t="n">
+      <c r="I214" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K214" s="5" t="n">
         <v>69.77</v>
       </c>
-      <c r="L214" s="33" t="inlineStr">
+      <c r="L214" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M214" s="32" t="n"/>
-      <c r="N214" s="34">
+      <c r="M214" s="2" t="n"/>
+      <c r="N214" s="4">
         <f>M214*G214</f>
         <v/>
       </c>
-      <c r="O214" s="32" t="n"/>
-      <c r="P214" s="32" t="n"/>
-      <c r="Q214" s="32" t="n"/>
-      <c r="R214" s="32" t="n"/>
-      <c r="S214" s="32" t="n"/>
+      <c r="O214" s="2" t="n"/>
+      <c r="P214" s="2" t="n"/>
+      <c r="Q214" s="2" t="n"/>
+      <c r="R214" s="2" t="n"/>
+      <c r="S214" s="2" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" s="32" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B215" s="32" t="n"/>
-      <c r="C215" s="33" t="inlineStr">
+      <c r="B215" s="2" t="n"/>
+      <c r="C215" s="3" t="inlineStr">
         <is>
           <t>Kolache Sausage Egg &amp; Cheese</t>
         </is>
       </c>
-      <c r="D215" s="33" t="n"/>
-      <c r="E215" s="32" t="n"/>
-      <c r="F215" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G215" s="34" t="n">
+      <c r="D215" s="3" t="n"/>
+      <c r="E215" s="2" t="n"/>
+      <c r="F215" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G215" s="4" t="n">
         <v>69.77</v>
       </c>
-      <c r="H215" s="35" t="n">
+      <c r="H215" s="5" t="n">
         <v>69.77</v>
       </c>
-      <c r="I215" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J215" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K215" s="35" t="n">
+      <c r="I215" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J215" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K215" s="5" t="n">
         <v>69.77</v>
       </c>
-      <c r="L215" s="33" t="inlineStr">
+      <c r="L215" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M215" s="32" t="n"/>
-      <c r="N215" s="34">
+      <c r="M215" s="2" t="n"/>
+      <c r="N215" s="4">
         <f>M215*G215</f>
         <v/>
       </c>
-      <c r="O215" s="32" t="n"/>
-      <c r="P215" s="32" t="n"/>
-      <c r="Q215" s="32" t="n"/>
-      <c r="R215" s="32" t="n"/>
-      <c r="S215" s="32" t="n"/>
+      <c r="O215" s="2" t="n"/>
+      <c r="P215" s="2" t="n"/>
+      <c r="Q215" s="2" t="n"/>
+      <c r="R215" s="2" t="n"/>
+      <c r="S215" s="2" t="n"/>
     </row>
     <row r="216">
-      <c r="A216" s="32" t="inlineStr">
+      <c r="A216" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B216" s="32" t="n"/>
-      <c r="C216" s="33" t="inlineStr">
+      <c r="B216" s="2" t="n"/>
+      <c r="C216" s="3" t="inlineStr">
         <is>
           <t>Wrap Jalapeno Popper</t>
         </is>
       </c>
-      <c r="D216" s="33" t="n"/>
-      <c r="E216" s="32" t="n"/>
-      <c r="F216" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G216" s="34" t="n">
+      <c r="D216" s="3" t="n"/>
+      <c r="E216" s="2" t="n"/>
+      <c r="F216" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G216" s="4" t="n">
         <v>93.03</v>
       </c>
-      <c r="H216" s="35" t="n">
+      <c r="H216" s="5" t="n">
         <v>93.03</v>
       </c>
-      <c r="I216" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J216" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K216" s="35" t="n">
+      <c r="I216" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J216" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K216" s="5" t="n">
         <v>93.03</v>
       </c>
-      <c r="L216" s="33" t="inlineStr">
+      <c r="L216" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M216" s="32" t="n"/>
-      <c r="N216" s="34">
+      <c r="M216" s="2" t="n"/>
+      <c r="N216" s="4">
         <f>M216*G216</f>
         <v/>
       </c>
-      <c r="O216" s="32" t="n"/>
-      <c r="P216" s="32" t="n"/>
-      <c r="Q216" s="32" t="n"/>
-      <c r="R216" s="32" t="n"/>
-      <c r="S216" s="32" t="n"/>
+      <c r="O216" s="2" t="n"/>
+      <c r="P216" s="2" t="n"/>
+      <c r="Q216" s="2" t="n"/>
+      <c r="R216" s="2" t="n"/>
+      <c r="S216" s="2" t="n"/>
     </row>
     <row r="217">
-      <c r="A217" s="32" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B217" s="32" t="n"/>
-      <c r="C217" s="33" t="inlineStr">
+      <c r="B217" s="2" t="n"/>
+      <c r="C217" s="3" t="inlineStr">
         <is>
           <t>Deer Burrito</t>
         </is>
       </c>
-      <c r="D217" s="33" t="n"/>
-      <c r="E217" s="32" t="n"/>
-      <c r="F217" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G217" s="34" t="n">
+      <c r="D217" s="3" t="n"/>
+      <c r="E217" s="2" t="n"/>
+      <c r="F217" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G217" s="4" t="n">
         <v>449</v>
       </c>
-      <c r="H217" s="35" t="n">
+      <c r="H217" s="5" t="n">
         <v>449</v>
       </c>
-      <c r="I217" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J217" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K217" s="35" t="n">
+      <c r="I217" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J217" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K217" s="5" t="n">
         <v>449</v>
       </c>
-      <c r="L217" s="33" t="inlineStr">
+      <c r="L217" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M217" s="32" t="n"/>
-      <c r="N217" s="34">
+      <c r="M217" s="2" t="n"/>
+      <c r="N217" s="4">
         <f>M217*G217</f>
         <v/>
       </c>
-      <c r="O217" s="32" t="n"/>
-      <c r="P217" s="32" t="n"/>
-      <c r="Q217" s="32" t="n"/>
-      <c r="R217" s="32" t="n"/>
-      <c r="S217" s="32" t="n"/>
+      <c r="O217" s="2" t="n"/>
+      <c r="P217" s="2" t="n"/>
+      <c r="Q217" s="2" t="n"/>
+      <c r="R217" s="2" t="n"/>
+      <c r="S217" s="2" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" s="32" t="inlineStr">
+      <c r="A218" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B218" s="32" t="n"/>
-      <c r="C218" s="33" t="inlineStr">
+      <c r="B218" s="2" t="n"/>
+      <c r="C218" s="3" t="inlineStr">
         <is>
           <t>Jalapeno Cheddar Kolache</t>
         </is>
       </c>
-      <c r="D218" s="33" t="n"/>
-      <c r="E218" s="32" t="n"/>
-      <c r="F218" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G218" s="34" t="n">
+      <c r="D218" s="3" t="n"/>
+      <c r="E218" s="2" t="n"/>
+      <c r="F218" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G218" s="4" t="n">
         <v>69.77</v>
       </c>
-      <c r="H218" s="35" t="n">
+      <c r="H218" s="5" t="n">
         <v>69.77</v>
       </c>
-      <c r="I218" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J218" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K218" s="35" t="n">
+      <c r="I218" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J218" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K218" s="5" t="n">
         <v>69.77</v>
       </c>
-      <c r="L218" s="33" t="inlineStr">
+      <c r="L218" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M218" s="32" t="n"/>
-      <c r="N218" s="34">
+      <c r="M218" s="2" t="n"/>
+      <c r="N218" s="4">
         <f>M218*G218</f>
         <v/>
       </c>
-      <c r="O218" s="32" t="n"/>
-      <c r="P218" s="32" t="n"/>
-      <c r="Q218" s="32" t="n"/>
-      <c r="R218" s="32" t="n"/>
-      <c r="S218" s="32" t="n"/>
+      <c r="O218" s="2" t="n"/>
+      <c r="P218" s="2" t="n"/>
+      <c r="Q218" s="2" t="n"/>
+      <c r="R218" s="2" t="n"/>
+      <c r="S218" s="2" t="n"/>
     </row>
     <row r="219">
-      <c r="A219" s="32" t="inlineStr">
+      <c r="A219" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B219" s="32" t="n"/>
-      <c r="C219" s="33" t="inlineStr">
+      <c r="B219" s="2" t="n"/>
+      <c r="C219" s="3" t="inlineStr">
         <is>
           <t>Chicken Fajita</t>
         </is>
       </c>
-      <c r="D219" s="33" t="n"/>
-      <c r="E219" s="32" t="n"/>
-      <c r="F219" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G219" s="34" t="n">
+      <c r="D219" s="3" t="n"/>
+      <c r="E219" s="2" t="n"/>
+      <c r="F219" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G219" s="4" t="n">
         <v>57.99</v>
       </c>
-      <c r="H219" s="35" t="n">
+      <c r="H219" s="5" t="n">
         <v>57.99</v>
       </c>
-      <c r="I219" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J219" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K219" s="35" t="n">
+      <c r="I219" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K219" s="5" t="n">
         <v>57.99</v>
       </c>
-      <c r="L219" s="33" t="inlineStr">
+      <c r="L219" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M219" s="32" t="n"/>
-      <c r="N219" s="34">
+      <c r="M219" s="2" t="n"/>
+      <c r="N219" s="4">
         <f>M219*G219</f>
         <v/>
       </c>
-      <c r="O219" s="32" t="n"/>
-      <c r="P219" s="32" t="n"/>
-      <c r="Q219" s="32" t="n"/>
-      <c r="R219" s="32" t="n"/>
-      <c r="S219" s="32" t="n"/>
+      <c r="O219" s="2" t="n"/>
+      <c r="P219" s="2" t="n"/>
+      <c r="Q219" s="2" t="n"/>
+      <c r="R219" s="2" t="n"/>
+      <c r="S219" s="2" t="n"/>
     </row>
     <row r="220">
-      <c r="A220" s="32" t="inlineStr">
+      <c r="A220" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B220" s="32" t="n"/>
-      <c r="C220" s="33" t="inlineStr">
+      <c r="B220" s="2" t="n"/>
+      <c r="C220" s="3" t="inlineStr">
         <is>
           <t>Mac And Cheese</t>
         </is>
       </c>
-      <c r="D220" s="33" t="n"/>
-      <c r="E220" s="32" t="inlineStr">
+      <c r="D220" s="3" t="n"/>
+      <c r="E220" s="2" t="inlineStr">
         <is>
           <t>6 Bags</t>
         </is>
       </c>
-      <c r="F220" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G220" s="34" t="n">
+      <c r="F220" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G220" s="4" t="n">
         <v>7.1</v>
       </c>
-      <c r="H220" s="35" t="n">
+      <c r="H220" s="5" t="n">
         <v>7.1</v>
       </c>
-      <c r="I220" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J220" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K220" s="35" t="n">
+      <c r="I220" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J220" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K220" s="5" t="n">
         <v>1.183333333333333</v>
       </c>
-      <c r="L220" s="33" t="inlineStr">
+      <c r="L220" s="3" t="inlineStr">
         <is>
           <t>per Bag (6 Bags)</t>
         </is>
       </c>
-      <c r="M220" s="32" t="n"/>
-      <c r="N220" s="34">
+      <c r="M220" s="2" t="n"/>
+      <c r="N220" s="4">
         <f>M220*G220</f>
         <v/>
       </c>
-      <c r="O220" s="32" t="n"/>
-      <c r="P220" s="32" t="n"/>
-      <c r="Q220" s="32" t="n"/>
-      <c r="R220" s="32" t="n"/>
-      <c r="S220" s="32" t="n"/>
+      <c r="O220" s="2" t="n"/>
+      <c r="P220" s="2" t="n"/>
+      <c r="Q220" s="2" t="n"/>
+      <c r="R220" s="2" t="n"/>
+      <c r="S220" s="2" t="n"/>
     </row>
     <row r="221">
-      <c r="A221" s="32" t="inlineStr">
+      <c r="A221" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B221" s="32" t="n"/>
-      <c r="C221" s="33" t="inlineStr">
+      <c r="B221" s="2" t="n"/>
+      <c r="C221" s="3" t="inlineStr">
         <is>
           <t>Mashed Potatoes</t>
         </is>
       </c>
-      <c r="D221" s="33" t="n"/>
-      <c r="E221" s="32" t="inlineStr">
+      <c r="D221" s="3" t="n"/>
+      <c r="E221" s="2" t="inlineStr">
         <is>
           <t>4 Bags</t>
         </is>
       </c>
-      <c r="F221" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G221" s="34" t="n">
+      <c r="F221" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G221" s="4" t="n">
         <v>9.640000000000001</v>
       </c>
-      <c r="H221" s="35" t="n">
+      <c r="H221" s="5" t="n">
         <v>9.640000000000001</v>
       </c>
-      <c r="I221" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J221" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K221" s="35" t="n">
+      <c r="I221" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J221" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K221" s="5" t="n">
         <v>2.41</v>
       </c>
-      <c r="L221" s="33" t="inlineStr">
+      <c r="L221" s="3" t="inlineStr">
         <is>
           <t>per Bag (4 Bags)</t>
         </is>
       </c>
-      <c r="M221" s="32" t="n"/>
-      <c r="N221" s="34">
+      <c r="M221" s="2" t="n"/>
+      <c r="N221" s="4">
         <f>M221*G221</f>
         <v/>
       </c>
-      <c r="O221" s="32" t="n"/>
-      <c r="P221" s="32" t="n"/>
-      <c r="Q221" s="32" t="n"/>
-      <c r="R221" s="32" t="n"/>
-      <c r="S221" s="32" t="n"/>
+      <c r="O221" s="2" t="n"/>
+      <c r="P221" s="2" t="n"/>
+      <c r="Q221" s="2" t="n"/>
+      <c r="R221" s="2" t="n"/>
+      <c r="S221" s="2" t="n"/>
     </row>
     <row r="222">
-      <c r="A222" s="32" t="inlineStr">
+      <c r="A222" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B222" s="32" t="n"/>
-      <c r="C222" s="33" t="inlineStr">
+      <c r="B222" s="2" t="n"/>
+      <c r="C222" s="3" t="inlineStr">
         <is>
           <t>Mini Taco Beef</t>
         </is>
       </c>
-      <c r="D222" s="33" t="n"/>
-      <c r="E222" s="32" t="inlineStr">
+      <c r="D222" s="3" t="n"/>
+      <c r="E222" s="2" t="inlineStr">
         <is>
           <t>case</t>
         </is>
       </c>
-      <c r="F222" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G222" s="34" t="n">
+      <c r="F222" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G222" s="4" t="n">
         <v>27.91</v>
       </c>
-      <c r="H222" s="35" t="n">
+      <c r="H222" s="5" t="n">
         <v>27.91</v>
       </c>
-      <c r="I222" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J222" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K222" s="35" t="n">
+      <c r="I222" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J222" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K222" s="5" t="n">
         <v>27.91</v>
       </c>
-      <c r="L222" s="33" t="inlineStr">
+      <c r="L222" s="3" t="inlineStr">
         <is>
           <t>per Case (case)</t>
         </is>
       </c>
-      <c r="M222" s="32" t="n"/>
-      <c r="N222" s="34">
+      <c r="M222" s="2" t="n"/>
+      <c r="N222" s="4">
         <f>M222*G222</f>
         <v/>
       </c>
-      <c r="O222" s="32" t="n"/>
-      <c r="P222" s="32" t="n"/>
-      <c r="Q222" s="32" t="n"/>
-      <c r="R222" s="32" t="n"/>
-      <c r="S222" s="32" t="n"/>
+      <c r="O222" s="2" t="n"/>
+      <c r="P222" s="2" t="n"/>
+      <c r="Q222" s="2" t="n"/>
+      <c r="R222" s="2" t="n"/>
+      <c r="S222" s="2" t="n"/>
     </row>
     <row r="223">
-      <c r="A223" s="32" t="inlineStr">
+      <c r="A223" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B223" s="32" t="n"/>
-      <c r="C223" s="33" t="inlineStr">
+      <c r="B223" s="2" t="n"/>
+      <c r="C223" s="3" t="inlineStr">
         <is>
           <t>Mini Taco Chicken</t>
         </is>
       </c>
-      <c r="D223" s="33" t="n"/>
-      <c r="E223" s="32" t="inlineStr">
+      <c r="D223" s="3" t="n"/>
+      <c r="E223" s="2" t="inlineStr">
         <is>
           <t>case</t>
         </is>
       </c>
-      <c r="F223" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G223" s="34" t="n">
+      <c r="F223" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G223" s="4" t="n">
         <v>27.91</v>
       </c>
-      <c r="H223" s="35" t="n">
+      <c r="H223" s="5" t="n">
         <v>27.91</v>
       </c>
-      <c r="I223" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J223" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K223" s="35" t="n">
+      <c r="I223" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J223" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K223" s="5" t="n">
         <v>27.91</v>
       </c>
-      <c r="L223" s="33" t="inlineStr">
+      <c r="L223" s="3" t="inlineStr">
         <is>
           <t>per Case (case)</t>
         </is>
       </c>
-      <c r="M223" s="32" t="n"/>
-      <c r="N223" s="34">
+      <c r="M223" s="2" t="n"/>
+      <c r="N223" s="4">
         <f>M223*G223</f>
         <v/>
       </c>
-      <c r="O223" s="32" t="n"/>
-      <c r="P223" s="32" t="n"/>
-      <c r="Q223" s="32" t="n"/>
-      <c r="R223" s="32" t="n"/>
-      <c r="S223" s="32" t="n"/>
+      <c r="O223" s="2" t="n"/>
+      <c r="P223" s="2" t="n"/>
+      <c r="Q223" s="2" t="n"/>
+      <c r="R223" s="2" t="n"/>
+      <c r="S223" s="2" t="n"/>
     </row>
     <row r="224">
-      <c r="A224" s="32" t="inlineStr">
+      <c r="A224" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B224" s="32" t="n"/>
-      <c r="C224" s="33" t="inlineStr">
+      <c r="B224" s="2" t="n"/>
+      <c r="C224" s="3" t="inlineStr">
         <is>
           <t>Red Beans</t>
         </is>
       </c>
-      <c r="D224" s="33" t="n"/>
-      <c r="E224" s="32" t="inlineStr">
+      <c r="D224" s="3" t="n"/>
+      <c r="E224" s="2" t="inlineStr">
         <is>
           <t>9 Bags</t>
         </is>
       </c>
-      <c r="F224" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G224" s="34" t="n">
+      <c r="F224" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G224" s="4" t="n">
         <v>6.49</v>
       </c>
-      <c r="H224" s="35" t="n">
+      <c r="H224" s="5" t="n">
         <v>6.49</v>
       </c>
-      <c r="I224" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J224" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K224" s="35" t="n">
+      <c r="I224" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J224" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K224" s="5" t="n">
         <v>0.7211111111111111</v>
       </c>
-      <c r="L224" s="33" t="inlineStr">
+      <c r="L224" s="3" t="inlineStr">
         <is>
           <t>per Bag (9 Bags)</t>
         </is>
       </c>
-      <c r="M224" s="32" t="n"/>
-      <c r="N224" s="34">
+      <c r="M224" s="2" t="n"/>
+      <c r="N224" s="4">
         <f>M224*G224</f>
         <v/>
       </c>
-      <c r="O224" s="32" t="n"/>
-      <c r="P224" s="32" t="n"/>
-      <c r="Q224" s="32" t="n"/>
-      <c r="R224" s="32" t="n"/>
-      <c r="S224" s="32" t="n"/>
+      <c r="O224" s="2" t="n"/>
+      <c r="P224" s="2" t="n"/>
+      <c r="Q224" s="2" t="n"/>
+      <c r="R224" s="2" t="n"/>
+      <c r="S224" s="2" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="32" t="inlineStr">
+      <c r="A225" s="2" t="inlineStr">
         <is>
           <t>PACK</t>
         </is>
       </c>
-      <c r="B225" s="32" t="n"/>
-      <c r="C225" s="33" t="inlineStr">
+      <c r="B225" s="2" t="n"/>
+      <c r="C225" s="3" t="inlineStr">
         <is>
           <t>Beef Sausage Dogs</t>
         </is>
       </c>
-      <c r="D225" s="33" t="n"/>
-      <c r="E225" s="32" t="n"/>
-      <c r="F225" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G225" s="34" t="n">
+      <c r="D225" s="3" t="n"/>
+      <c r="E225" s="2" t="n"/>
+      <c r="F225" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G225" s="4" t="n">
         <v>20.34</v>
       </c>
-      <c r="H225" s="35" t="n">
+      <c r="H225" s="5" t="n">
         <v>20.34</v>
       </c>
-      <c r="I225" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J225" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K225" s="35" t="n">
+      <c r="I225" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J225" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K225" s="5" t="n">
         <v>20.34</v>
       </c>
-      <c r="L225" s="33" t="inlineStr">
+      <c r="L225" s="3" t="inlineStr">
         <is>
           <t>per Pack (None)</t>
         </is>
       </c>
-      <c r="M225" s="32" t="n"/>
-      <c r="N225" s="34">
+      <c r="M225" s="2" t="n"/>
+      <c r="N225" s="4">
         <f>M225*G225</f>
         <v/>
       </c>
-      <c r="O225" s="32" t="n"/>
-      <c r="P225" s="32" t="n"/>
-      <c r="Q225" s="32" t="n"/>
-      <c r="R225" s="32" t="n"/>
-      <c r="S225" s="32" t="n"/>
+      <c r="O225" s="2" t="n"/>
+      <c r="P225" s="2" t="n"/>
+      <c r="Q225" s="2" t="n"/>
+      <c r="R225" s="2" t="n"/>
+      <c r="S225" s="2" t="n"/>
     </row>
     <row r="226">
-      <c r="A226" s="32" t="inlineStr">
+      <c r="A226" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B226" s="32" t="n"/>
-      <c r="C226" s="33" t="inlineStr">
+      <c r="B226" s="2" t="n"/>
+      <c r="C226" s="3" t="inlineStr">
         <is>
           <t>Seasoned Corn</t>
         </is>
       </c>
-      <c r="D226" s="33" t="n"/>
-      <c r="E226" s="32" t="inlineStr">
+      <c r="D226" s="3" t="n"/>
+      <c r="E226" s="2" t="inlineStr">
         <is>
           <t>6 Bags</t>
         </is>
       </c>
-      <c r="F226" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G226" s="34" t="n">
+      <c r="F226" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G226" s="4" t="n">
         <v>6.18</v>
       </c>
-      <c r="H226" s="35" t="n">
+      <c r="H226" s="5" t="n">
         <v>6.18</v>
       </c>
-      <c r="I226" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J226" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K226" s="35" t="n">
+      <c r="I226" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K226" s="5" t="n">
         <v>1.03</v>
       </c>
-      <c r="L226" s="33" t="inlineStr">
+      <c r="L226" s="3" t="inlineStr">
         <is>
           <t>per Bag (6 Bags)</t>
         </is>
       </c>
-      <c r="M226" s="32" t="n"/>
-      <c r="N226" s="34">
+      <c r="M226" s="2" t="n"/>
+      <c r="N226" s="4">
         <f>M226*G226</f>
         <v/>
       </c>
-      <c r="O226" s="32" t="n"/>
-      <c r="P226" s="32" t="n"/>
-      <c r="Q226" s="32" t="n"/>
-      <c r="R226" s="32" t="n"/>
-      <c r="S226" s="32" t="n"/>
+      <c r="O226" s="2" t="n"/>
+      <c r="P226" s="2" t="n"/>
+      <c r="Q226" s="2" t="n"/>
+      <c r="R226" s="2" t="n"/>
+      <c r="S226" s="2" t="n"/>
     </row>
     <row r="227">
-      <c r="A227" s="32" t="inlineStr">
+      <c r="A227" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B227" s="32" t="n"/>
-      <c r="C227" s="33" t="inlineStr">
+      <c r="B227" s="2" t="n"/>
+      <c r="C227" s="3" t="inlineStr">
         <is>
           <t>Stuffed Nacho</t>
         </is>
       </c>
-      <c r="D227" s="33" t="n"/>
-      <c r="E227" s="32" t="inlineStr">
+      <c r="D227" s="3" t="n"/>
+      <c r="E227" s="2" t="inlineStr">
         <is>
           <t>case</t>
         </is>
       </c>
-      <c r="F227" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G227" s="34" t="n">
+      <c r="F227" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G227" s="4" t="n">
         <v>37.28</v>
       </c>
-      <c r="H227" s="35" t="n">
+      <c r="H227" s="5" t="n">
         <v>37.28</v>
       </c>
-      <c r="I227" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J227" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K227" s="35" t="n">
+      <c r="I227" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J227" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K227" s="5" t="n">
         <v>37.28</v>
       </c>
-      <c r="L227" s="33" t="inlineStr">
+      <c r="L227" s="3" t="inlineStr">
         <is>
           <t>per Case (case)</t>
         </is>
       </c>
-      <c r="M227" s="32" t="n"/>
-      <c r="N227" s="34">
+      <c r="M227" s="2" t="n"/>
+      <c r="N227" s="4">
         <f>M227*G227</f>
         <v/>
       </c>
-      <c r="O227" s="32" t="n"/>
-      <c r="P227" s="32" t="n"/>
-      <c r="Q227" s="32" t="n"/>
-      <c r="R227" s="32" t="n"/>
-      <c r="S227" s="32" t="n"/>
+      <c r="O227" s="2" t="n"/>
+      <c r="P227" s="2" t="n"/>
+      <c r="Q227" s="2" t="n"/>
+      <c r="R227" s="2" t="n"/>
+      <c r="S227" s="2" t="n"/>
     </row>
     <row r="228">
-      <c r="A228" s="32" t="inlineStr">
+      <c r="A228" s="2" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="B228" s="32" t="n"/>
-      <c r="C228" s="33" t="inlineStr">
+      <c r="B228" s="2" t="n"/>
+      <c r="C228" s="3" t="inlineStr">
         <is>
           <t>Tomato Gravy</t>
         </is>
       </c>
-      <c r="D228" s="33" t="n"/>
-      <c r="E228" s="32" t="inlineStr">
+      <c r="D228" s="3" t="n"/>
+      <c r="E228" s="2" t="inlineStr">
         <is>
           <t>4 bags</t>
         </is>
       </c>
-      <c r="F228" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G228" s="34" t="n">
+      <c r="F228" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G228" s="4" t="n">
         <v>12.34</v>
       </c>
-      <c r="H228" s="35" t="n">
+      <c r="H228" s="5" t="n">
         <v>12.34</v>
       </c>
-      <c r="I228" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J228" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K228" s="35" t="n">
+      <c r="I228" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K228" s="5" t="n">
         <v>3.085</v>
       </c>
-      <c r="L228" s="33" t="inlineStr">
+      <c r="L228" s="3" t="inlineStr">
         <is>
           <t>per Bag (4 bags)</t>
         </is>
       </c>
-      <c r="M228" s="32" t="n"/>
-      <c r="N228" s="34">
+      <c r="M228" s="2" t="n"/>
+      <c r="N228" s="4">
         <f>M228*G228</f>
         <v/>
       </c>
-      <c r="O228" s="32" t="n"/>
-      <c r="P228" s="32" t="n"/>
-      <c r="Q228" s="32" t="n"/>
-      <c r="R228" s="32" t="n"/>
-      <c r="S228" s="32" t="n"/>
+      <c r="O228" s="2" t="n"/>
+      <c r="P228" s="2" t="n"/>
+      <c r="Q228" s="2" t="n"/>
+      <c r="R228" s="2" t="n"/>
+      <c r="S228" s="2" t="n"/>
     </row>
     <row r="229">
-      <c r="A229" s="32" t="inlineStr">
+      <c r="A229" s="2" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="B229" s="32" t="n"/>
-      <c r="C229" s="33" t="inlineStr">
+      <c r="B229" s="2" t="n"/>
+      <c r="C229" s="3" t="inlineStr">
         <is>
           <t>Spicy Chicken Patty</t>
         </is>
       </c>
-      <c r="D229" s="33" t="n"/>
-      <c r="E229" s="32" t="n"/>
-      <c r="F229" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G229" s="34" t="n">
+      <c r="D229" s="3" t="n"/>
+      <c r="E229" s="2" t="n"/>
+      <c r="F229" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G229" s="4" t="n">
         <v>52.87</v>
       </c>
-      <c r="H229" s="35" t="n">
+      <c r="H229" s="5" t="n">
         <v>52.87</v>
       </c>
-      <c r="I229" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J229" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K229" s="35" t="n">
+      <c r="I229" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K229" s="5" t="n">
         <v>52.87</v>
       </c>
-      <c r="L229" s="33" t="inlineStr">
+      <c r="L229" s="3" t="inlineStr">
         <is>
           <t>per Case (None)</t>
         </is>
       </c>
-      <c r="M229" s="32" t="n"/>
-      <c r="N229" s="34">
+      <c r="M229" s="2" t="n"/>
+      <c r="N229" s="4">
         <f>M229*G229</f>
         <v/>
       </c>
-      <c r="O229" s="32" t="n"/>
-      <c r="P229" s="32" t="n"/>
-      <c r="Q229" s="32" t="n"/>
-      <c r="R229" s="32" t="n"/>
-      <c r="S229" s="32" t="n"/>
+      <c r="O229" s="2" t="n"/>
+      <c r="P229" s="2" t="n"/>
+      <c r="Q229" s="2" t="n"/>
+      <c r="R229" s="2" t="n"/>
+      <c r="S229" s="2" t="n"/>
     </row>
     <row r="230">
-      <c r="A230" s="32" t="inlineStr">
+      <c r="A230" s="2" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B230" s="32" t="n"/>
-      <c r="C230" s="33" t="inlineStr">
+      <c r="B230" s="2" t="n"/>
+      <c r="C230" s="3" t="inlineStr">
         <is>
           <t>Crooked Letter Cookies</t>
         </is>
       </c>
-      <c r="D230" s="33" t="n"/>
-      <c r="E230" s="32" t="n"/>
-      <c r="F230" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G230" s="34" t="n">
+      <c r="D230" s="3" t="n"/>
+      <c r="E230" s="2" t="n"/>
+      <c r="F230" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G230" s="4" t="n">
         <v>1.9</v>
       </c>
-      <c r="H230" s="35" t="n">
+      <c r="H230" s="5" t="n">
         <v>1.9</v>
       </c>
-      <c r="I230" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J230" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K230" s="35" t="n">
+      <c r="I230" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K230" s="5" t="n">
         <v>1.9</v>
       </c>
-      <c r="L230" s="33" t="inlineStr">
+      <c r="L230" s="3" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M230" s="32" t="n"/>
-      <c r="N230" s="34">
+      <c r="M230" s="2" t="n"/>
+      <c r="N230" s="4">
         <f>M230*G230</f>
         <v/>
       </c>
-      <c r="O230" s="32" t="n"/>
-      <c r="P230" s="32" t="n"/>
-      <c r="Q230" s="32" t="n"/>
-      <c r="R230" s="32" t="n"/>
-      <c r="S230" s="32" t="n"/>
+      <c r="O230" s="2" t="n"/>
+      <c r="P230" s="2" t="n"/>
+      <c r="Q230" s="2" t="n"/>
+      <c r="R230" s="2" t="n"/>
+      <c r="S230" s="2" t="n"/>
     </row>
     <row r="231">
-      <c r="A231" s="32" t="inlineStr">
+      <c r="A231" s="2" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B231" s="32" t="n"/>
-      <c r="C231" s="33" t="inlineStr">
+      <c r="B231" s="2" t="n"/>
+      <c r="C231" s="3" t="inlineStr">
         <is>
           <t>Strawberry/Blueberry Cream Cheese King Cake</t>
         </is>
       </c>
-      <c r="D231" s="33" t="n"/>
-      <c r="E231" s="32" t="n"/>
-      <c r="F231" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G231" s="34" t="n">
+      <c r="D231" s="3" t="n"/>
+      <c r="E231" s="2" t="n"/>
+      <c r="F231" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G231" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="H231" s="35" t="n">
+      <c r="H231" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="I231" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J231" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K231" s="35" t="n">
+      <c r="I231" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K231" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="L231" s="33" t="inlineStr">
+      <c r="L231" s="3" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M231" s="32" t="n"/>
-      <c r="N231" s="34">
+      <c r="M231" s="2" t="n"/>
+      <c r="N231" s="4">
         <f>M231*G231</f>
         <v/>
       </c>
-      <c r="O231" s="32" t="n"/>
-      <c r="P231" s="32" t="n"/>
-      <c r="Q231" s="32" t="n"/>
-      <c r="R231" s="32" t="n"/>
-      <c r="S231" s="32" t="n"/>
+      <c r="O231" s="2" t="n"/>
+      <c r="P231" s="2" t="n"/>
+      <c r="Q231" s="2" t="n"/>
+      <c r="R231" s="2" t="n"/>
+      <c r="S231" s="2" t="n"/>
     </row>
     <row r="232">
-      <c r="A232" s="32" t="inlineStr">
+      <c r="A232" s="2" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B232" s="32" t="n"/>
-      <c r="C232" s="33" t="inlineStr">
+      <c r="B232" s="2" t="n"/>
+      <c r="C232" s="3" t="inlineStr">
         <is>
           <t>Traditional King Cake</t>
         </is>
       </c>
-      <c r="D232" s="33" t="n"/>
-      <c r="E232" s="32" t="n"/>
-      <c r="F232" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G232" s="34" t="n">
+      <c r="D232" s="3" t="n"/>
+      <c r="E232" s="2" t="n"/>
+      <c r="F232" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G232" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="H232" s="35" t="n">
+      <c r="H232" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="I232" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J232" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K232" s="35" t="n">
+      <c r="I232" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K232" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="L232" s="33" t="inlineStr">
+      <c r="L232" s="3" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M232" s="32" t="n"/>
-      <c r="N232" s="34">
+      <c r="M232" s="2" t="n"/>
+      <c r="N232" s="4">
         <f>M232*G232</f>
         <v/>
       </c>
-      <c r="O232" s="32" t="n"/>
-      <c r="P232" s="32" t="n"/>
-      <c r="Q232" s="32" t="n"/>
-      <c r="R232" s="32" t="n"/>
-      <c r="S232" s="32" t="n"/>
+      <c r="O232" s="2" t="n"/>
+      <c r="P232" s="2" t="n"/>
+      <c r="Q232" s="2" t="n"/>
+      <c r="R232" s="2" t="n"/>
+      <c r="S232" s="2" t="n"/>
     </row>
     <row r="233">
-      <c r="A233" s="32" t="inlineStr">
+      <c r="A233" s="2" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B233" s="32" t="n"/>
-      <c r="C233" s="33" t="inlineStr">
+      <c r="B233" s="2" t="n"/>
+      <c r="C233" s="3" t="inlineStr">
         <is>
           <t>Cream Cheese King Cake</t>
         </is>
       </c>
-      <c r="D233" s="33" t="n"/>
-      <c r="E233" s="32" t="n"/>
-      <c r="F233" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G233" s="34" t="n">
+      <c r="D233" s="3" t="n"/>
+      <c r="E233" s="2" t="n"/>
+      <c r="F233" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G233" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="H233" s="35" t="n">
+      <c r="H233" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="I233" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J233" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K233" s="35" t="n">
+      <c r="I233" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="L233" s="33" t="inlineStr">
+      <c r="L233" s="3" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M233" s="32" t="n"/>
-      <c r="N233" s="34">
+      <c r="M233" s="2" t="n"/>
+      <c r="N233" s="4">
         <f>M233*G233</f>
         <v/>
       </c>
-      <c r="O233" s="32" t="n"/>
-      <c r="P233" s="32" t="n"/>
-      <c r="Q233" s="32" t="n"/>
-      <c r="R233" s="32" t="n"/>
-      <c r="S233" s="32" t="n"/>
+      <c r="O233" s="2" t="n"/>
+      <c r="P233" s="2" t="n"/>
+      <c r="Q233" s="2" t="n"/>
+      <c r="R233" s="2" t="n"/>
+      <c r="S233" s="2" t="n"/>
     </row>
     <row r="234">
-      <c r="A234" s="32" t="inlineStr">
+      <c r="A234" s="2" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="B234" s="32" t="n"/>
-      <c r="C234" s="33" t="inlineStr">
+      <c r="B234" s="2" t="n"/>
+      <c r="C234" s="3" t="inlineStr">
         <is>
           <t>Pecan Praline King Cake</t>
         </is>
       </c>
-      <c r="D234" s="33" t="n"/>
-      <c r="E234" s="32" t="n"/>
-      <c r="F234" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G234" s="34" t="n">
+      <c r="D234" s="3" t="n"/>
+      <c r="E234" s="2" t="n"/>
+      <c r="F234" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G234" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="H234" s="35" t="n">
+      <c r="H234" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="I234" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J234" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K234" s="35" t="n">
+      <c r="I234" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="L234" s="33" t="inlineStr">
+      <c r="L234" s="3" t="inlineStr">
         <is>
           <t>per Each (None)</t>
         </is>
       </c>
-      <c r="M234" s="32" t="n"/>
-      <c r="N234" s="34">
+      <c r="M234" s="2" t="n"/>
+      <c r="N234" s="4">
         <f>M234*G234</f>
         <v/>
       </c>
-      <c r="O234" s="32" t="n"/>
-      <c r="P234" s="32" t="n"/>
-      <c r="Q234" s="32" t="n"/>
-      <c r="R234" s="32" t="n"/>
-      <c r="S234" s="32" t="n"/>
+      <c r="O234" s="2" t="n"/>
+      <c r="P234" s="2" t="n"/>
+      <c r="Q234" s="2" t="n"/>
+      <c r="R234" s="2" t="n"/>
+      <c r="S234" s="2" t="n"/>
     </row>
     <row r="236">
-      <c r="A236" s="38" t="inlineStr">
+      <c r="A236" s="35" t="inlineStr">
         <is>
           <t>COLOR LEGEND</t>
         </is>
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="33" t="inlineStr">
-        <is>
-          <t>DARK RED   — No BEK item number (not in BEK list)</t>
-        </is>
-      </c>
-      <c r="B237" s="39" t="n"/>
-      <c r="C237" s="39" t="n"/>
-      <c r="D237" s="39" t="n"/>
+      <c r="A237" s="27" t="inlineStr">
+        <is>
+          <t>RED    — No matching BEK item number (needs manual lookup)</t>
+        </is>
+      </c>
+      <c r="B237" s="36" t="n"/>
+      <c r="C237" s="36" t="n"/>
+      <c r="D237" s="36" t="n"/>
     </row>
     <row r="238">
-      <c r="A238" s="27" t="inlineStr">
-        <is>
-          <t>ORANGE-RED — BEK# not found in current price list</t>
-        </is>
-      </c>
-      <c r="B238" s="39" t="n"/>
-      <c r="C238" s="39" t="n"/>
-      <c r="D238" s="39" t="n"/>
+      <c r="A238" s="21" t="inlineStr">
+        <is>
+          <t>PINK   — Price UP ≥ 10% or ≥ $2.00/unit</t>
+        </is>
+      </c>
+      <c r="B238" s="36" t="n"/>
+      <c r="C238" s="36" t="n"/>
+      <c r="D238" s="36" t="n"/>
     </row>
     <row r="239">
-      <c r="A239" s="21" t="inlineStr">
-        <is>
-          <t>PINK       — Price UP ≥ 10% or ≥ $2.00/unit</t>
-        </is>
-      </c>
-      <c r="B239" s="39" t="n"/>
-      <c r="C239" s="39" t="n"/>
-      <c r="D239" s="39" t="n"/>
+      <c r="A239" s="15" t="inlineStr">
+        <is>
+          <t>YELLOW — Price increased (under threshold)</t>
+        </is>
+      </c>
+      <c r="B239" s="36" t="n"/>
+      <c r="C239" s="36" t="n"/>
+      <c r="D239" s="36" t="n"/>
     </row>
     <row r="240">
-      <c r="A240" s="15" t="inlineStr">
-        <is>
-          <t>YELLOW     — Price increased (under threshold)</t>
-        </is>
-      </c>
-      <c r="B240" s="39" t="n"/>
-      <c r="C240" s="39" t="n"/>
-      <c r="D240" s="39" t="n"/>
+      <c r="A240" s="9" t="inlineStr">
+        <is>
+          <t>GREEN  — Price decreased</t>
+        </is>
+      </c>
+      <c r="B240" s="36" t="n"/>
+      <c r="C240" s="36" t="n"/>
+      <c r="D240" s="36" t="n"/>
     </row>
     <row r="241">
-      <c r="A241" s="9" t="inlineStr">
-        <is>
-          <t>GREEN      — Price decreased</t>
-        </is>
-      </c>
-      <c r="B241" s="39" t="n"/>
-      <c r="C241" s="39" t="n"/>
-      <c r="D241" s="39" t="n"/>
-    </row>
-    <row r="242">
-      <c r="A242" s="3" t="inlineStr">
-        <is>
-          <t>WHITE      — No change / price matched</t>
-        </is>
-      </c>
-      <c r="B242" s="39" t="n"/>
-      <c r="C242" s="39" t="n"/>
-      <c r="D242" s="39" t="n"/>
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>WHITE  — No change / BEK match confirmed</t>
+        </is>
+      </c>
+      <c r="B241" s="36" t="n"/>
+      <c r="C241" s="36" t="n"/>
+      <c r="D241" s="36" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A202:S202"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13816,795 +13833,795 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="40" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>PRODUCT</t>
         </is>
       </c>
-      <c r="B1" s="40" t="inlineStr">
+      <c r="B1" s="37" t="inlineStr">
         <is>
           <t>SIZE/DESCRIPTION</t>
         </is>
       </c>
-      <c r="C1" s="40" t="inlineStr">
+      <c r="C1" s="37" t="inlineStr">
         <is>
           <t>ON HAND (QTY)</t>
         </is>
       </c>
-      <c r="D1" s="40" t="inlineStr">
+      <c r="D1" s="37" t="inlineStr">
         <is>
           <t>COST</t>
         </is>
       </c>
-      <c r="E1" s="40" t="inlineStr">
+      <c r="E1" s="37" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="41" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>SIGNATURE BLEND</t>
         </is>
       </c>
-      <c r="B2" s="41" t="inlineStr">
+      <c r="B2" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C2" s="42" t="n">
+      <c r="C2" s="39" t="n">
         <v>1.5</v>
       </c>
-      <c r="D2" s="42" t="n"/>
-      <c r="E2" s="42" t="n"/>
+      <c r="D2" s="39" t="n"/>
+      <c r="E2" s="39" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="41" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>AMERICAN CLASSIC</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C3" s="42" t="n">
+      <c r="C3" s="39" t="n">
         <v>1.75</v>
       </c>
-      <c r="D3" s="42" t="n"/>
-      <c r="E3" s="42" t="n"/>
+      <c r="D3" s="39" t="n"/>
+      <c r="E3" s="39" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="41" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>PECAN PRALINE</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C4" s="42" t="n">
+      <c r="C4" s="39" t="n">
         <v>1.5</v>
       </c>
-      <c r="D4" s="42" t="n"/>
-      <c r="E4" s="42" t="n"/>
+      <c r="D4" s="39" t="n"/>
+      <c r="E4" s="39" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="41" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>BREAKFAST BLEND</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C5" s="42" t="n">
+      <c r="C5" s="39" t="n">
         <v>1.75</v>
       </c>
-      <c r="D5" s="42" t="n"/>
-      <c r="E5" s="42" t="n"/>
+      <c r="D5" s="39" t="n"/>
+      <c r="E5" s="39" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="41" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>DB ESPRESSO</t>
         </is>
       </c>
-      <c r="B6" s="41" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C6" s="42" t="n">
+      <c r="C6" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="42" t="n"/>
-      <c r="E6" s="42" t="n"/>
+      <c r="D6" s="39" t="n"/>
+      <c r="E6" s="39" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="41" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>Creamer Cups (Irish Cream, French Vanilla, Caramel)</t>
         </is>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C7" s="42" t="n">
+      <c r="C7" s="39" t="n">
         <v>3.5</v>
       </c>
-      <c r="D7" s="42" t="n"/>
-      <c r="E7" s="42" t="n"/>
+      <c r="D7" s="39" t="n"/>
+      <c r="E7" s="39" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="41" t="inlineStr">
+      <c r="A8" s="38" t="inlineStr">
         <is>
           <t>Coffee Mate</t>
         </is>
       </c>
-      <c r="B8" s="41" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C8" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="42" t="n"/>
-      <c r="E8" s="42" t="n"/>
+      <c r="C8" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="39" t="n"/>
+      <c r="E8" s="39" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="41" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>Sweet Cream Creamer</t>
         </is>
       </c>
-      <c r="B9" s="41" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C9" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="42" t="n"/>
-      <c r="E9" s="42" t="n"/>
+      <c r="C9" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="41" t="inlineStr">
+      <c r="A10" s="38" t="inlineStr">
         <is>
           <t>Hazelnut Creamer</t>
         </is>
       </c>
-      <c r="B10" s="41" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C10" s="42" t="n">
+      <c r="C10" s="39" t="n">
         <v>1.1</v>
       </c>
-      <c r="D10" s="42" t="n"/>
-      <c r="E10" s="42" t="n"/>
+      <c r="D10" s="39" t="n"/>
+      <c r="E10" s="39" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="41" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>Half And Half</t>
         </is>
       </c>
-      <c r="B11" s="41" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C11" s="42" t="n">
+      <c r="C11" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="42" t="n"/>
-      <c r="E11" s="42" t="n"/>
+      <c r="D11" s="39" t="n"/>
+      <c r="E11" s="39" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="41" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>Original Creamer</t>
         </is>
       </c>
-      <c r="B12" s="41" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C12" s="42" t="n">
+      <c r="C12" s="39" t="n">
         <v>1.25</v>
       </c>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="42" t="n"/>
+      <c r="D12" s="39" t="n"/>
+      <c r="E12" s="39" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="41" t="inlineStr">
+      <c r="A13" s="38" t="inlineStr">
         <is>
           <t>Caramel Syrup Pump</t>
         </is>
       </c>
-      <c r="B13" s="41" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>BOTTLE</t>
         </is>
       </c>
-      <c r="C13" s="42" t="n">
+      <c r="C13" s="39" t="n">
         <v>1.5</v>
       </c>
-      <c r="D13" s="42" t="n"/>
-      <c r="E13" s="42" t="n"/>
+      <c r="D13" s="39" t="n"/>
+      <c r="E13" s="39" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="41" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>Hazelnut Syrup Pump</t>
         </is>
       </c>
-      <c r="B14" s="41" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>BOTTLE</t>
         </is>
       </c>
-      <c r="C14" s="42" t="n">
+      <c r="C14" s="39" t="n">
         <v>1.5</v>
       </c>
-      <c r="D14" s="42" t="n"/>
-      <c r="E14" s="42" t="n"/>
+      <c r="D14" s="39" t="n"/>
+      <c r="E14" s="39" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="41" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>French Vanilla Syrup Pump</t>
         </is>
       </c>
-      <c r="B15" s="41" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>BOTTLE</t>
         </is>
       </c>
-      <c r="C15" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="42" t="n"/>
-      <c r="E15" s="42" t="n"/>
+      <c r="C15" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="39" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>Hold &amp; Go Lids 12-24oz</t>
         </is>
       </c>
-      <c r="B16" s="41" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="C16" s="42" t="n">
+      <c r="C16" s="39" t="n">
         <v>14</v>
       </c>
-      <c r="D16" s="42" t="n"/>
-      <c r="E16" s="42" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="39" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="41" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>Lid SW 16/20oz</t>
         </is>
       </c>
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="C17" s="42" t="n"/>
-      <c r="D17" s="42" t="n"/>
-      <c r="E17" s="42" t="n"/>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="39" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="41" t="inlineStr">
+      <c r="A18" s="38" t="inlineStr">
         <is>
           <t>Cappuccino French Vanilla</t>
         </is>
       </c>
-      <c r="B18" s="41" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C18" s="42" t="n">
+      <c r="C18" s="39" t="n">
         <v>9</v>
       </c>
-      <c r="D18" s="42" t="n"/>
-      <c r="E18" s="42" t="n"/>
+      <c r="D18" s="39" t="n"/>
+      <c r="E18" s="39" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>Sugar Free Cappuccino French Vanilla</t>
         </is>
       </c>
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C19" s="42" t="n">
+      <c r="C19" s="39" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="42" t="n"/>
-      <c r="E19" s="42" t="n"/>
+      <c r="D19" s="39" t="n"/>
+      <c r="E19" s="39" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="41" t="inlineStr">
+      <c r="A20" s="38" t="inlineStr">
         <is>
           <t>Hot Chocolate</t>
         </is>
       </c>
-      <c r="B20" s="41" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C20" s="42" t="n">
+      <c r="C20" s="39" t="n">
         <v>11</v>
       </c>
-      <c r="D20" s="42" t="n"/>
-      <c r="E20" s="42" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="39" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="41" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>Creamer Packs</t>
         </is>
       </c>
-      <c r="B21" s="41" t="inlineStr">
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C21" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="42" t="n"/>
-      <c r="E21" s="42" t="n"/>
+      <c r="C21" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="39" t="n"/>
+      <c r="E21" s="39" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>Sugar Pack</t>
         </is>
       </c>
-      <c r="B22" s="41" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C22" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="42" t="n"/>
-      <c r="E22" s="42" t="n"/>
+      <c r="C22" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="39" t="n"/>
+      <c r="E22" s="39" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="41" t="inlineStr">
+      <c r="A23" s="38" t="inlineStr">
         <is>
           <t>Blue Sweetener</t>
         </is>
       </c>
-      <c r="B23" s="41" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C23" s="42" t="n">
+      <c r="C23" s="39" t="n">
         <v>0.75</v>
       </c>
-      <c r="D23" s="42" t="n"/>
-      <c r="E23" s="42" t="n"/>
+      <c r="D23" s="39" t="n"/>
+      <c r="E23" s="39" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="41" t="inlineStr">
+      <c r="A24" s="38" t="inlineStr">
         <is>
           <t>Yellow Sweetener</t>
         </is>
       </c>
-      <c r="B24" s="41" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>CASE</t>
         </is>
       </c>
-      <c r="C24" s="42" t="n">
+      <c r="C24" s="39" t="n">
         <v>0.25</v>
       </c>
-      <c r="D24" s="42" t="n"/>
-      <c r="E24" s="42" t="n"/>
+      <c r="D24" s="39" t="n"/>
+      <c r="E24" s="39" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="41" t="inlineStr">
+      <c r="A25" s="38" t="inlineStr">
         <is>
           <t>Pink Sweetener</t>
         </is>
       </c>
-      <c r="B25" s="41" t="inlineStr">
+      <c r="B25" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C25" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="42" t="n"/>
-      <c r="E25" s="42" t="n"/>
+      <c r="C25" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="39" t="n"/>
+      <c r="E25" s="39" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="41" t="inlineStr">
+      <c r="A26" s="38" t="inlineStr">
         <is>
           <t>Sugar Packets</t>
         </is>
       </c>
-      <c r="B26" s="41" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="C26" s="42" t="n">
+      <c r="C26" s="39" t="n">
         <v>45</v>
       </c>
-      <c r="D26" s="42" t="n"/>
-      <c r="E26" s="42" t="n"/>
+      <c r="D26" s="39" t="n"/>
+      <c r="E26" s="39" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="41" t="inlineStr">
+      <c r="A27" s="38" t="inlineStr">
         <is>
           <t>Sugar Canister</t>
         </is>
       </c>
-      <c r="B27" s="41" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="C27" s="42" t="n">
+      <c r="C27" s="39" t="n">
         <v>39</v>
       </c>
-      <c r="D27" s="42" t="n"/>
-      <c r="E27" s="42" t="n"/>
+      <c r="D27" s="39" t="n"/>
+      <c r="E27" s="39" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="41" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>Red Stirrers</t>
         </is>
       </c>
-      <c r="B28" s="41" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>PACK</t>
         </is>
       </c>
-      <c r="C28" s="42" t="n">
+      <c r="C28" s="39" t="n">
         <v>3.5</v>
       </c>
-      <c r="D28" s="42" t="n"/>
-      <c r="E28" s="42" t="n"/>
+      <c r="D28" s="39" t="n"/>
+      <c r="E28" s="39" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="41" t="inlineStr">
+      <c r="A29" s="38" t="inlineStr">
         <is>
           <t>16 oz Double-Wall Cup</t>
         </is>
       </c>
-      <c r="B29" s="41" t="inlineStr">
+      <c r="B29" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C29" s="42" t="n">
+      <c r="C29" s="39" t="n">
         <v>32</v>
       </c>
-      <c r="D29" s="42" t="n"/>
-      <c r="E29" s="42" t="n"/>
+      <c r="D29" s="39" t="n"/>
+      <c r="E29" s="39" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="41" t="inlineStr">
+      <c r="A30" s="38" t="inlineStr">
         <is>
           <t>16oz Single-Wall Cup</t>
         </is>
       </c>
-      <c r="B30" s="41" t="inlineStr">
+      <c r="B30" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C30" s="42" t="n"/>
-      <c r="D30" s="42" t="n"/>
-      <c r="E30" s="42" t="n"/>
+      <c r="C30" s="39" t="n"/>
+      <c r="D30" s="39" t="n"/>
+      <c r="E30" s="39" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="41" t="inlineStr">
+      <c r="A31" s="38" t="inlineStr">
         <is>
           <t>24 oz Double-Wall Cup</t>
         </is>
       </c>
-      <c r="B31" s="41" t="inlineStr">
+      <c r="B31" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C31" s="42" t="n">
+      <c r="C31" s="39" t="n">
         <v>37</v>
       </c>
-      <c r="D31" s="42" t="n"/>
-      <c r="E31" s="42" t="n"/>
+      <c r="D31" s="39" t="n"/>
+      <c r="E31" s="39" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="41" t="inlineStr">
+      <c r="A32" s="38" t="inlineStr">
         <is>
           <t>32oz Fountain Cup</t>
         </is>
       </c>
-      <c r="B32" s="41" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C32" s="42" t="n">
+      <c r="C32" s="39" t="n">
         <v>63</v>
       </c>
-      <c r="D32" s="42" t="n"/>
-      <c r="E32" s="42" t="n"/>
+      <c r="D32" s="39" t="n"/>
+      <c r="E32" s="39" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="41" t="inlineStr">
+      <c r="A33" s="38" t="inlineStr">
         <is>
           <t>32oz Lid</t>
         </is>
       </c>
-      <c r="B33" s="41" t="inlineStr">
+      <c r="B33" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C33" s="42" t="n">
+      <c r="C33" s="39" t="n">
         <v>61</v>
       </c>
-      <c r="D33" s="43" t="n">
+      <c r="D33" s="40" t="n">
         <v>2.85</v>
       </c>
-      <c r="E33" s="43">
+      <c r="E33" s="40">
         <f>C33*D33</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="41" t="inlineStr">
+      <c r="A34" s="38" t="inlineStr">
         <is>
           <t>20oz Cup</t>
         </is>
       </c>
-      <c r="B34" s="41" t="inlineStr">
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C34" s="42" t="n">
+      <c r="C34" s="39" t="n">
         <v>81</v>
       </c>
-      <c r="D34" s="42" t="n"/>
-      <c r="E34" s="42" t="n"/>
+      <c r="D34" s="39" t="n"/>
+      <c r="E34" s="39" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="41" t="inlineStr">
+      <c r="A35" s="38" t="inlineStr">
         <is>
           <t>20oz Lid</t>
         </is>
       </c>
-      <c r="B35" s="41" t="inlineStr">
+      <c r="B35" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C35" s="42" t="n">
+      <c r="C35" s="39" t="n">
         <v>56</v>
       </c>
-      <c r="D35" s="42" t="n"/>
-      <c r="E35" s="42" t="n"/>
+      <c r="D35" s="39" t="n"/>
+      <c r="E35" s="39" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="41" t="inlineStr">
+      <c r="A36" s="38" t="inlineStr">
         <is>
           <t>Red Straws</t>
         </is>
       </c>
-      <c r="B36" s="41" t="inlineStr">
+      <c r="B36" s="38" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="C36" s="42" t="n">
+      <c r="C36" s="39" t="n">
         <v>12</v>
       </c>
-      <c r="D36" s="42" t="n"/>
-      <c r="E36" s="42" t="n"/>
+      <c r="D36" s="39" t="n"/>
+      <c r="E36" s="39" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="41" t="inlineStr">
+      <c r="A37" s="38" t="inlineStr">
         <is>
           <t>Bag In Box 5 Gal Syrup</t>
         </is>
       </c>
-      <c r="B37" s="41" t="inlineStr">
+      <c r="B37" s="38" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="C37" s="42" t="n">
+      <c r="C37" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="D37" s="42" t="n"/>
-      <c r="E37" s="42" t="n"/>
+      <c r="D37" s="39" t="n"/>
+      <c r="E37" s="39" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="41" t="inlineStr">
+      <c r="A38" s="38" t="inlineStr">
         <is>
           <t>Bag In Box 2.5 Gal Syrup</t>
         </is>
       </c>
-      <c r="B38" s="41" t="inlineStr">
+      <c r="B38" s="38" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="C38" s="42" t="n">
+      <c r="C38" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="D38" s="42" t="n"/>
-      <c r="E38" s="42" t="n"/>
+      <c r="D38" s="39" t="n"/>
+      <c r="E38" s="39" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="41" t="inlineStr">
+      <c r="A39" s="38" t="inlineStr">
         <is>
           <t>CO2 Tank</t>
         </is>
       </c>
-      <c r="B39" s="41" t="inlineStr">
+      <c r="B39" s="38" t="inlineStr">
         <is>
           <t>EACH</t>
         </is>
       </c>
-      <c r="C39" s="42" t="n">
+      <c r="C39" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="D39" s="42" t="n"/>
-      <c r="E39" s="42" t="n"/>
+      <c r="D39" s="39" t="n"/>
+      <c r="E39" s="39" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="41" t="inlineStr">
+      <c r="A40" s="38" t="inlineStr">
         <is>
           <t>Cafe Tango Lids</t>
         </is>
       </c>
-      <c r="B40" s="41" t="inlineStr">
+      <c r="B40" s="38" t="inlineStr">
         <is>
           <t>SLEEVE</t>
         </is>
       </c>
-      <c r="C40" s="42" t="n">
+      <c r="C40" s="39" t="n">
         <v>6</v>
       </c>
-      <c r="D40" s="43" t="n">
+      <c r="D40" s="40" t="n">
         <v>2.53</v>
       </c>
-      <c r="E40" s="43">
+      <c r="E40" s="40">
         <f>C40*D40</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="41" t="inlineStr">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>16 oz Tango Cup</t>
         </is>
       </c>
-      <c r="B41" s="41" t="inlineStr">
+      <c r="B41" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C41" s="42" t="n">
+      <c r="C41" s="39" t="n">
         <v>8</v>
       </c>
-      <c r="D41" s="43" t="n">
+      <c r="D41" s="40" t="n">
         <v>6.78</v>
       </c>
-      <c r="E41" s="43">
+      <c r="E41" s="40">
         <f>C41*D41</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="41" t="inlineStr">
+      <c r="A42" s="38" t="inlineStr">
         <is>
           <t>24 oz Tango Cup</t>
         </is>
       </c>
-      <c r="B42" s="41" t="inlineStr">
+      <c r="B42" s="38" t="inlineStr">
         <is>
           <t>SLV</t>
         </is>
       </c>
-      <c r="C42" s="42" t="n">
+      <c r="C42" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="D42" s="42" t="n"/>
-      <c r="E42" s="42" t="n"/>
+      <c r="D42" s="39" t="n"/>
+      <c r="E42" s="39" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="41" t="inlineStr">
+      <c r="A43" s="38" t="inlineStr">
         <is>
           <t>Cafe Tango French Vanilla</t>
         </is>
       </c>
-      <c r="B43" s="41" t="inlineStr">
+      <c r="B43" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C43" s="42" t="n">
+      <c r="C43" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="D43" s="43" t="n">
+      <c r="D43" s="40" t="n">
         <v>13.64</v>
       </c>
-      <c r="E43" s="43">
+      <c r="E43" s="40">
         <f>C43*D43</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="41" t="inlineStr">
+      <c r="A44" s="38" t="inlineStr">
         <is>
           <t>Cafe Tango Mocha</t>
         </is>
       </c>
-      <c r="B44" s="41" t="inlineStr">
+      <c r="B44" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C44" s="42" t="n">
+      <c r="C44" s="39" t="n">
         <v>25</v>
       </c>
-      <c r="D44" s="42" t="n"/>
-      <c r="E44" s="42" t="n"/>
+      <c r="D44" s="39" t="n"/>
+      <c r="E44" s="39" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="41" t="inlineStr">
+      <c r="A45" s="38" t="inlineStr">
         <is>
           <t>Caramel Macchiato</t>
         </is>
       </c>
-      <c r="B45" s="41" t="inlineStr">
+      <c r="B45" s="38" t="inlineStr">
         <is>
           <t>BAG</t>
         </is>
       </c>
-      <c r="C45" s="42" t="n">
+      <c r="C45" s="39" t="n">
         <v>14</v>
       </c>
-      <c r="D45" s="42" t="n"/>
-      <c r="E45" s="42" t="n"/>
+      <c r="D45" s="39" t="n"/>
+      <c r="E45" s="39" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>